<commit_message>
Add ambiguity review sheet to the real-world dataset
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01McHC4aiqYXQ7NJ1sbfn4HC
</commit_message>
<xml_diff>
--- a/dataset/sqli_real_dataset.xlsx
+++ b/dataset/sqli_real_dataset.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="real_rows" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="blank_columns" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ambiguity_review" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -46812,4 +46813,1696 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D76"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>pair (vulnerable id)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>what is ambiguous</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>suggested action</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>real_0186</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A. fixed row still vulnerable</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>The label-0 version still builds SQL from input: real_0187 keeps "page_name = '%s'" % page_name, real_0217 keeps an f-string IN list.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Relabel the fixed row to 1 or drop the pair</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>real_0216</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>A. fixed row still vulnerable</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>The label-0 version still builds SQL from input: real_0187 keeps "page_name = '%s'" % page_name, real_0217 keeps an f-string IN list.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Relabel the fixed row to 1 or drop the pair</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>real_0242</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>B. vulnerable row not vulnerable</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>The before version already used placeholders; the commit is a refactor.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Drop the pair</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>real_0000</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>B. vulnerable only through %d / %i</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>The value is formatted with %d or %i, which forces a number, so text cannot break the query. Bad practice but arguably not injectable.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Keep as label 1, move to a separate case type, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>real_0008</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>B. vulnerable only through %d / %i</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>The value is formatted with %d or %i, which forces a number, so text cannot break the query. Bad practice but arguably not injectable.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Keep as label 1, move to a separate case type, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>real_0060</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>B. vulnerable only through %d / %i</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>The value is formatted with %d or %i, which forces a number, so text cannot break the query. Bad practice but arguably not injectable.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Keep as label 1, move to a separate case type, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>real_0104</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>B. vulnerable only through %d / %i</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>The value is formatted with %d or %i, which forces a number, so text cannot break the query. Bad practice but arguably not injectable.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Keep as label 1, move to a separate case type, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>real_0128</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>B. vulnerable only through %d / %i</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>The value is formatted with %d or %i, which forces a number, so text cannot break the query. Bad practice but arguably not injectable.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Keep as label 1, move to a separate case type, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>real_0154</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>B. vulnerable only through %d / %i</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>The value is formatted with %d or %i, which forces a number, so text cannot break the query. Bad practice but arguably not injectable.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Keep as label 1, move to a separate case type, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>real_0198</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>B. vulnerable only through %d / %i</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>The value is formatted with %d or %i, which forces a number, so text cannot break the query. Bad practice but arguably not injectable.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Keep as label 1, move to a separate case type, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>real_0304</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>B. vulnerable only through %d / %i</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>The value is formatted with %d or %i, which forces a number, so text cannot break the query. Bad practice but arguably not injectable.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Keep as label 1, move to a separate case type, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>real_0306</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>B. vulnerable only through %d / %i</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>The value is formatted with %d or %i, which forces a number, so text cannot break the query. Bad practice but arguably not injectable.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Keep as label 1, move to a separate case type, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>real_0310</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>B. vulnerable only through %d / %i</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>The value is formatted with %d or %i, which forces a number, so text cannot break the query. Bad practice but arguably not injectable.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Keep as label 1, move to a separate case type, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>real_0330</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>B. vulnerable only through %d / %i</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>The value is formatted with %d or %i, which forces a number, so text cannot break the query. Bad practice but arguably not injectable.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Keep as label 1, move to a separate case type, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>real_0332</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>B. vulnerable only through %d / %i</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>The value is formatted with %d or %i, which forces a number, so text cannot break the query. Bad practice but arguably not injectable.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Keep as label 1, move to a separate case type, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>real_0350</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>B. vulnerable only through %d / %i</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>The value is formatted with %d or %i, which forces a number, so text cannot break the query. Bad practice but arguably not injectable.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Keep as label 1, move to a separate case type, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>real_0360</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>B. vulnerable only through %d / %i</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>The value is formatted with %d or %i, which forces a number, so text cannot break the query. Bad practice but arguably not injectable.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Keep as label 1, move to a separate case type, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>real_0368</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>B. vulnerable only through %d / %i</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>The value is formatted with %d or %i, which forces a number, so text cannot break the query. Bad practice but arguably not injectable.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Keep as label 1, move to a separate case type, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>real_0372</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>B. vulnerable only through %d / %i</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>The value is formatted with %d or %i, which forces a number, so text cannot break the query. Bad practice but arguably not injectable.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Keep as label 1, move to a separate case type, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>real_0386</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>B. vulnerable only through %d / %i</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>The value is formatted with %d or %i, which forces a number, so text cannot break the query. Bad practice but arguably not injectable.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Keep as label 1, move to a separate case type, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>real_0042</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>C. fix does not work</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>The fix uses a placeholder for a table name, which the driver rejects.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Keep code as label 1 but treat fixed_code as invalid, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>real_0106</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>C. fix does not work</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>The fix uses a placeholder for a table name, which the driver rejects.</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Keep code as label 1 but treat fixed_code as invalid, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>real_0302</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>C. fix does not work</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>The fix uses a placeholder for a table name, which the driver rejects.</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Keep code as label 1 but treat fixed_code as invalid, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>real_0210</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>C. fix does not work</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>The fix uses a placeholder for a table name, which the driver rejects.</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Keep code as label 1 but treat fixed_code as invalid, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>real_0238</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>C. fix does not work</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Fixed code is missing a comma before the parameter tuple, so it raises at runtime.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Repair the comma or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>real_0124</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>C. fix does not work</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Placeholders are wrapped in quotes or use %d, which these drivers reject or store with extra quotes.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Repair the placeholders or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>real_0148</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>C. fix does not work</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Placeholders are wrapped in quotes or use %d, which these drivers reject or store with extra quotes.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Repair the placeholders or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>real_0214</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>C. fix does not work</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Placeholders are wrapped in quotes or use %d, which these drivers reject or store with extra quotes.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Repair the placeholders or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>real_0028</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>C. fix does not work</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>The parameter is passed as a bare string or number instead of a tuple; sqlite3 fails unless it is one character long.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Repair to a one-element tuple or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>real_0060</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>C. fix does not work</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>The parameter is passed as a bare string or number instead of a tuple; sqlite3 fails unless it is one character long.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Repair to a one-element tuple or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>real_0076</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>C. fix does not work</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>The parameter is passed as a bare string or number instead of a tuple; sqlite3 fails unless it is one character long.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Repair to a one-element tuple or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>real_0112</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>C. fix does not work</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>The parameter is passed as a bare string or number instead of a tuple; sqlite3 fails unless it is one character long.</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Repair to a one-element tuple or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>real_0304</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>C. fix does not work</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>The parameter is passed as a bare string or number instead of a tuple; sqlite3 fails unless it is one character long.</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Repair to a one-element tuple or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>real_0332</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>C. fix does not work</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>The parameter is passed as a bare string or number instead of a tuple; sqlite3 fails unless it is one character long.</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Repair to a one-element tuple or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>real_0342</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>C. fix does not work</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>The parameter is passed as a bare string or number instead of a tuple; sqlite3 fails unless it is one character long.</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Repair to a one-element tuple or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>real_0002</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>D. fix depends on an unseen wrapper</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>The fix keeps '{name}' inside quotes and passes a dict to a project-specific db.exec(); whether that is actually safe depends on code that is not in the row.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Keep with a note, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>real_0016</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>D. fix depends on an unseen wrapper</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>The fix keeps '{name}' inside quotes and passes a dict to a project-specific db.exec(); whether that is actually safe depends on code that is not in the row.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Keep with a note, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>real_0038</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>D. fix depends on an unseen wrapper</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>The fix keeps '{name}' inside quotes and passes a dict to a project-specific db.exec(); whether that is actually safe depends on code that is not in the row.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Keep with a note, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>real_0094</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>D. fix depends on an unseen wrapper</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>The fix keeps '{name}' inside quotes and passes a dict to a project-specific db.exec(); whether that is actually safe depends on code that is not in the row.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Keep with a note, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>real_0142</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>D. fix depends on an unseen wrapper</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>The fix keeps '{name}' inside quotes and passes a dict to a project-specific db.exec(); whether that is actually safe depends on code that is not in the row.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Keep with a note, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>real_0160</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>D. fix depends on an unseen wrapper</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>The fix keeps '{name}' inside quotes and passes a dict to a project-specific db.exec(); whether that is actually safe depends on code that is not in the row.</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Keep with a note, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>real_0192</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>D. fix depends on an unseen wrapper</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>The fix keeps '{name}' inside quotes and passes a dict to a project-specific db.exec(); whether that is actually safe depends on code that is not in the row.</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Keep with a note, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>real_0244</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>D. fix depends on an unseen wrapper</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>The fix keeps '{name}' inside quotes and passes a dict to a project-specific db.exec(); whether that is actually safe depends on code that is not in the row.</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Keep with a note, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>real_0286</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>D. fix depends on an unseen wrapper</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>The fix keeps '{name}' inside quotes and passes a dict to a project-specific db.exec(); whether that is actually safe depends on code that is not in the row.</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Keep with a note, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>real_0298</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>D. fix depends on an unseen wrapper</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>The fix keeps '{name}' inside quotes and passes a dict to a project-specific db.exec(); whether that is actually safe depends on code that is not in the row.</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Keep with a note, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>real_0322</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>D. fix depends on an unseen wrapper</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>The fix keeps '{name}' inside quotes and passes a dict to a project-specific db.exec(); whether that is actually safe depends on code that is not in the row.</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Keep with a note, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>real_0346</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>D. fix depends on an unseen wrapper</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>The fix keeps '{name}' inside quotes and passes a dict to a project-specific db.exec(); whether that is actually safe depends on code that is not in the row.</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Keep with a note, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>real_0348</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>D. fix depends on an unseen wrapper</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>The fix keeps '{name}' inside quotes and passes a dict to a project-specific db.exec(); whether that is actually safe depends on code that is not in the row.</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Keep with a note, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>real_0376</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>D. fix depends on an unseen wrapper</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>The fix keeps '{name}' inside quotes and passes a dict to a project-specific db.exec(); whether that is actually safe depends on code that is not in the row.</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Keep with a note, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>real_0004</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>D. fix depends on an unseen wrapper</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>self.query(q, value) passes one bare value; correct only if the wrapper wraps it in a tuple.</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Keep with a note</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>real_0020</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>D. fix depends on an unseen wrapper</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>self.query(q, value) passes one bare value; correct only if the wrapper wraps it in a tuple.</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Keep with a note</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>real_0056</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>D. fix depends on an unseen wrapper</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>self.query(q, value) passes one bare value; correct only if the wrapper wraps it in a tuple.</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Keep with a note</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>real_0276</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>D. fix depends on an unseen wrapper</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>self.query(q, value) passes one bare value; correct only if the wrapper wraps it in a tuple.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Keep with a note</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>real_0232</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>E. fix is partial</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>The fix still formats the column name mType from the caller into SET %s.</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Relabel fixed row as still weak, or drop</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>real_0010</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>E. fixed row formats a table name</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>The table name comes from config or self.table (trusted), values use placeholders. Fine, but a scanner will still flag it.</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Keep as label 0 (hard-negative style)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>real_0078</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>E. fixed row formats a table name</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>The table name comes from config or self.table (trusted), values use placeholders. Fine, but a scanner will still flag it.</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Keep as label 0 (hard-negative style)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>real_0206</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>E. fixed row formats a table name</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>The table name comes from config or self.table (trusted), values use placeholders. Fine, but a scanner will still flag it.</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Keep as label 0 (hard-negative style)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>real_0246</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>E. fixed row formats a table name</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>The table name comes from config or self.table (trusted), values use placeholders. Fine, but a scanner will still flag it.</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Keep as label 0 (hard-negative style)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>real_0324</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>E. fixed row formats a table name</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>The table name comes from config or self.table (trusted), values use placeholders. Fine, but a scanner will still flag it.</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Keep as label 0 (hard-negative style)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>real_0404</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>E. fixed row formats a table name</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>The table name comes from config or self.table (trusted), values use placeholders. Fine, but a scanner will still flag it.</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Keep as label 0 (hard-negative style)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>real_0082</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>E. fixed row formats a table name</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>The table name comes from config or self.table (trusted), values use placeholders. Fine, but a scanner will still flag it.</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Keep as label 0 (hard-negative style)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>real_0118</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>E. fixed row formats a table name</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>The table name comes from config or self.table (trusted), values use placeholders. Fine, but a scanner will still flag it.</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Keep as label 0 (hard-negative style)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>real_0166</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>E. fixed row formats a table name</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>The table name comes from config or self.table (trusted), values use placeholders. Fine, but a scanner will still flag it.</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Keep as label 0 (hard-negative style)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>real_0268</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>E. fixed row formats a table name</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>The table name comes from config or self.table (trusted), values use placeholders. Fine, but a scanner will still flag it.</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Keep as label 0 (hard-negative style)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>real_0080</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>F. diff has unrelated changes</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>The commit also changes lines that have nothing to do with the SQL.</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Keep; vulnerable_lines may include extra lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>real_0152</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>F. diff has unrelated changes</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>The commit also changes lines that have nothing to do with the SQL.</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Keep; vulnerable_lines may include extra lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>real_0160</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>F. diff has unrelated changes</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>The commit also changes lines that have nothing to do with the SQL.</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Keep; vulnerable_lines may include extra lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>real_0194</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>F. diff has unrelated changes</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>The commit also changes lines that have nothing to do with the SQL.</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Keep; vulnerable_lines may include extra lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>real_0144 (+0176,0196,0252,0266,0402)</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>G. near-duplicates</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>37 pairs in 13 groups have the same code shape after renaming, mostly from the same repository.</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Keep one per group</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>real_0026 (+0034,0224,0398)</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>G. near-duplicates</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>37 pairs in 13 groups have the same code shape after renaming, mostly from the same repository.</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Keep one per group</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>real_0306 (+0310,0330,0368)</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>G. near-duplicates</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>37 pairs in 13 groups have the same code shape after renaming, mostly from the same repository.</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Keep one per group</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>real_0008 (+0104,0360)</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>G. near-duplicates</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>37 pairs in 13 groups have the same code shape after renaming, mostly from the same repository.</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Keep one per group</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>real_0062 (+0248,0394)</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>G. near-duplicates</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>37 pairs in 13 groups have the same code shape after renaming, mostly from the same repository.</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Keep one per group</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>real_0130 (+0256,0296)</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>G. near-duplicates</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>37 pairs in 13 groups have the same code shape after renaming, mostly from the same repository.</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Keep one per group</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>+7 more pairs of 2</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>G. near-duplicates</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>37 pairs in 13 groups have the same code shape after renaming, mostly from the same repository.</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Keep one per group</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>